<commit_message>
Update MSFT financial model
</commit_message>
<xml_diff>
--- a/NBIS Model.xlsx
+++ b/NBIS Model.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kerem\OneDrive\Masaüstü\Models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDF126A8-CBA2-42FB-8998-F9F2F46A1D83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87B16C55-4552-4DE1-89F9-E3DA4695BCDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25260" yWindow="360" windowWidth="27216" windowHeight="16248" xr2:uid="{15DD2EF7-3D38-48BE-91C3-905AF47E584F}"/>
+    <workbookView xWindow="4416" yWindow="0" windowWidth="21384" windowHeight="16200" xr2:uid="{15DD2EF7-3D38-48BE-91C3-905AF47E584F}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -37,14 +37,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="112">
   <si>
     <t>Company Overview</t>
   </si>
   <si>
-    <t>Recommendation:</t>
-  </si>
-  <si>
     <t>Target:</t>
   </si>
   <si>
@@ -313,9 +310,6 @@
   </si>
   <si>
     <t>Avride Stake</t>
-  </si>
-  <si>
-    <t>Hold</t>
   </si>
   <si>
     <t>Q3 25</t>
@@ -468,18 +462,12 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -530,7 +518,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -554,19 +542,16 @@
     <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="37" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -589,7 +574,7 @@
     <xf numFmtId="37" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="8" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -597,18 +582,13 @@
     <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="8" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="5" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -633,10 +613,15 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1049,540 +1034,536 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="46" t="s">
-        <v>94</v>
-      </c>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
+      <c r="B2" s="55"/>
+      <c r="C2" s="55"/>
+      <c r="D2" s="56" t="s">
+        <v>92</v>
+      </c>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B3" s="45"/>
-      <c r="C3" s="45"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
-      <c r="H3" s="13" t="s">
+      <c r="B3" s="55"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="56"/>
+      <c r="E3" s="56"/>
+      <c r="F3" s="56"/>
+      <c r="H3" s="13"/>
+      <c r="J3" s="13"/>
+      <c r="L3" s="13" t="s">
         <v>1</v>
-      </c>
-      <c r="J3" s="19" t="s">
-        <v>92</v>
-      </c>
-      <c r="L3" s="13" t="s">
-        <v>2</v>
       </c>
       <c r="M3" s="1">
         <v>119.64</v>
       </c>
       <c r="O3" s="13" t="s">
-        <v>43</v>
-      </c>
-      <c r="Q3" s="20" t="s">
-        <v>93</v>
+        <v>42</v>
+      </c>
+      <c r="Q3" s="19" t="s">
+        <v>91</v>
       </c>
       <c r="R3" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="S3" s="51">
+        <v>18</v>
+      </c>
+      <c r="S3" s="47">
         <v>46037</v>
       </c>
-      <c r="T3" s="51"/>
+      <c r="T3" s="47"/>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B4" s="45"/>
-      <c r="C4" s="45"/>
-      <c r="D4" s="46"/>
-      <c r="E4" s="46"/>
-      <c r="F4" s="46"/>
+      <c r="B4" s="55"/>
+      <c r="C4" s="55"/>
+      <c r="D4" s="56"/>
+      <c r="E4" s="56"/>
+      <c r="F4" s="56"/>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B5" s="21" t="s">
+      <c r="B5" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="21"/>
-      <c r="D5" s="22"/>
-      <c r="E5" s="22"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="22"/>
-      <c r="I5" s="22"/>
-      <c r="J5" s="22"/>
-      <c r="K5" s="22"/>
-      <c r="L5" s="22"/>
-      <c r="M5" s="22"/>
-      <c r="N5" s="22"/>
-      <c r="O5" s="22"/>
-      <c r="P5" s="22"/>
-      <c r="Q5" s="22"/>
-      <c r="R5" s="22"/>
-      <c r="S5" s="22"/>
-      <c r="T5" s="22"/>
-      <c r="U5" s="40"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="21"/>
+      <c r="H5" s="21"/>
+      <c r="I5" s="21"/>
+      <c r="J5" s="21"/>
+      <c r="K5" s="21"/>
+      <c r="L5" s="21"/>
+      <c r="M5" s="21"/>
+      <c r="N5" s="21"/>
+      <c r="O5" s="21"/>
+      <c r="P5" s="21"/>
+      <c r="Q5" s="21"/>
+      <c r="R5" s="21"/>
+      <c r="S5" s="21"/>
+      <c r="T5" s="21"/>
+      <c r="U5" s="39"/>
     </row>
     <row r="6" spans="1:21" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
-      <c r="B6" s="47" t="s">
+      <c r="B6" s="57" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" s="57"/>
+      <c r="D6" s="57"/>
+      <c r="E6" s="57"/>
+      <c r="F6" s="57"/>
+      <c r="H6" s="57" t="s">
+        <v>7</v>
+      </c>
+      <c r="I6" s="57"/>
+      <c r="J6" s="57"/>
+      <c r="K6" s="57"/>
+      <c r="L6" s="57"/>
+      <c r="M6" s="57"/>
+      <c r="O6" s="57" t="s">
+        <v>12</v>
+      </c>
+      <c r="P6" s="57"/>
+      <c r="Q6" s="57"/>
+      <c r="R6" s="22" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="B7" s="54" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="47"/>
-      <c r="D6" s="47"/>
-      <c r="E6" s="47"/>
-      <c r="F6" s="47"/>
-      <c r="H6" s="47" t="s">
+      <c r="C7" s="54"/>
+      <c r="D7" s="50" t="s">
+        <v>93</v>
+      </c>
+      <c r="E7" s="51"/>
+      <c r="F7" s="51"/>
+      <c r="H7" s="54" t="s">
         <v>8</v>
       </c>
-      <c r="I6" s="47"/>
-      <c r="J6" s="47"/>
-      <c r="K6" s="47"/>
-      <c r="L6" s="47"/>
-      <c r="M6" s="47"/>
-      <c r="O6" s="47" t="s">
+      <c r="I7" s="54"/>
+      <c r="J7" s="48">
+        <v>1371</v>
+      </c>
+      <c r="K7" s="48"/>
+      <c r="L7" s="48"/>
+      <c r="M7" s="48"/>
+      <c r="O7" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="P6" s="47"/>
-      <c r="Q6" s="47"/>
-      <c r="R6" s="23" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B7" s="48" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" s="48"/>
-      <c r="D7" s="54" t="s">
-        <v>95</v>
-      </c>
-      <c r="E7" s="55"/>
-      <c r="F7" s="55"/>
-      <c r="H7" s="48" t="s">
-        <v>9</v>
-      </c>
-      <c r="I7" s="48"/>
-      <c r="J7" s="52">
-        <v>1371</v>
-      </c>
-      <c r="K7" s="52"/>
-      <c r="L7" s="52"/>
-      <c r="M7" s="52"/>
-      <c r="O7" s="1" t="s">
-        <v>14</v>
       </c>
       <c r="R7" s="11">
         <v>87.41</v>
       </c>
-      <c r="S7" s="24"/>
-      <c r="T7" s="24"/>
+      <c r="S7" s="23"/>
+      <c r="T7" s="23"/>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B8" s="45" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="45"/>
-      <c r="D8" s="56">
-        <v>103.89</v>
-      </c>
-      <c r="E8" s="56"/>
-      <c r="F8" s="56"/>
-      <c r="H8" s="45" t="s">
-        <v>10</v>
-      </c>
-      <c r="I8" s="45"/>
-      <c r="J8" s="53">
+      <c r="B8" s="55" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="55"/>
+      <c r="D8" s="52">
+        <v>70</v>
+      </c>
+      <c r="E8" s="52"/>
+      <c r="F8" s="52"/>
+      <c r="H8" s="55" t="s">
+        <v>9</v>
+      </c>
+      <c r="I8" s="55"/>
+      <c r="J8" s="49">
         <v>2000</v>
       </c>
-      <c r="K8" s="53"/>
-      <c r="L8" s="53"/>
-      <c r="M8" s="53"/>
+      <c r="K8" s="49"/>
+      <c r="L8" s="49"/>
+      <c r="M8" s="49"/>
       <c r="O8" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="R8" s="11">
         <v>259</v>
       </c>
-      <c r="S8" s="24"/>
-      <c r="T8" s="24"/>
+      <c r="S8" s="23"/>
+      <c r="T8" s="23"/>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B9" s="45" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="45"/>
-      <c r="D9" s="56">
+      <c r="B9" s="55" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="55"/>
+      <c r="D9" s="52">
         <f>N54/R8</f>
-        <v>119.63526866771996</v>
-      </c>
-      <c r="E9" s="56"/>
-      <c r="F9" s="56"/>
-      <c r="H9" s="45" t="s">
-        <v>11</v>
-      </c>
-      <c r="I9" s="45"/>
-      <c r="J9" s="53" t="s">
-        <v>96</v>
-      </c>
-      <c r="K9" s="53"/>
-      <c r="L9" s="53"/>
-      <c r="M9" s="53"/>
+        <v>102.39055573940966</v>
+      </c>
+      <c r="E9" s="52"/>
+      <c r="F9" s="52"/>
+      <c r="H9" s="55" t="s">
+        <v>10</v>
+      </c>
+      <c r="I9" s="55"/>
+      <c r="J9" s="49" t="s">
+        <v>94</v>
+      </c>
+      <c r="K9" s="49"/>
+      <c r="L9" s="49"/>
+      <c r="M9" s="49"/>
       <c r="O9" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="R9" s="11">
         <f>-4795-107.1+4091+405.4</f>
         <v>-405.70000000000039</v>
       </c>
-      <c r="S9" s="28"/>
-      <c r="T9" s="28"/>
+      <c r="S9" s="27"/>
+      <c r="T9" s="27"/>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B10" s="45" t="s">
-        <v>7</v>
-      </c>
-      <c r="C10" s="45"/>
-      <c r="D10" s="50">
+      <c r="B10" s="55" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="55"/>
+      <c r="D10" s="46">
         <f>D9/D8-1</f>
-        <v>0.15155711490730539</v>
-      </c>
-      <c r="E10" s="50"/>
-      <c r="F10" s="50"/>
-      <c r="H10" s="45" t="s">
-        <v>12</v>
-      </c>
-      <c r="I10" s="45"/>
-      <c r="J10" s="53" t="s">
-        <v>97</v>
-      </c>
-      <c r="K10" s="53"/>
-      <c r="L10" s="53"/>
-      <c r="M10" s="53"/>
+        <v>0.46272222484870951</v>
+      </c>
+      <c r="E10" s="46"/>
+      <c r="F10" s="46"/>
+      <c r="H10" s="55" t="s">
+        <v>11</v>
+      </c>
+      <c r="I10" s="55"/>
+      <c r="J10" s="49" t="s">
+        <v>95</v>
+      </c>
+      <c r="K10" s="49"/>
+      <c r="L10" s="49"/>
+      <c r="M10" s="49"/>
       <c r="O10" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="R10" s="11">
         <f>R7*R8+R9</f>
         <v>22233.489999999998</v>
       </c>
-      <c r="S10" s="24"/>
-      <c r="T10" s="24"/>
+      <c r="S10" s="23"/>
+      <c r="T10" s="23"/>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B11" s="45"/>
-      <c r="C11" s="45"/>
-      <c r="D11" s="50"/>
-      <c r="E11" s="50"/>
-      <c r="F11" s="50"/>
-      <c r="H11" s="45"/>
-      <c r="I11" s="45"/>
-      <c r="J11" s="57"/>
-      <c r="K11" s="57"/>
-      <c r="L11" s="57"/>
-      <c r="M11" s="57"/>
-      <c r="S11" s="29"/>
-      <c r="T11" s="29"/>
+      <c r="B11" s="55"/>
+      <c r="C11" s="55"/>
+      <c r="D11" s="46"/>
+      <c r="E11" s="46"/>
+      <c r="F11" s="46"/>
+      <c r="H11" s="55"/>
+      <c r="I11" s="55"/>
+      <c r="J11" s="53"/>
+      <c r="K11" s="53"/>
+      <c r="L11" s="53"/>
+      <c r="M11" s="53"/>
+      <c r="S11" s="28"/>
+      <c r="T11" s="28"/>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B12" s="21" t="s">
-        <v>61</v>
-      </c>
-      <c r="C12" s="21"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="21">
+      <c r="B12" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="C12" s="20"/>
+      <c r="D12" s="21"/>
+      <c r="E12" s="20">
         <v>2020</v>
       </c>
-      <c r="F12" s="21">
+      <c r="F12" s="20">
         <v>2021</v>
       </c>
-      <c r="G12" s="21">
+      <c r="G12" s="20">
         <v>2022</v>
       </c>
-      <c r="H12" s="21">
+      <c r="H12" s="20">
         <v>2023</v>
       </c>
-      <c r="I12" s="21">
+      <c r="I12" s="20">
         <v>2024</v>
       </c>
-      <c r="J12" s="25" t="s">
-        <v>76</v>
-      </c>
-      <c r="K12" s="25" t="s">
+      <c r="J12" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="K12" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="L12" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="L12" s="25" t="s">
+      <c r="M12" s="24" t="s">
         <v>55</v>
       </c>
-      <c r="M12" s="25" t="s">
+      <c r="N12" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="N12" s="25" t="s">
+      <c r="O12" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="O12" s="25" t="s">
-        <v>58</v>
-      </c>
-      <c r="P12" s="25" t="s">
+      <c r="P12" s="24" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q12" s="24" t="s">
         <v>71</v>
       </c>
-      <c r="Q12" s="25" t="s">
+      <c r="R12" s="24" t="s">
         <v>72</v>
       </c>
-      <c r="R12" s="25" t="s">
+      <c r="S12" s="24" t="s">
         <v>73</v>
       </c>
-      <c r="S12" s="25" t="s">
+      <c r="T12" s="24" t="s">
         <v>74</v>
-      </c>
-      <c r="T12" s="25" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B13" s="13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C13" s="13"/>
       <c r="D13" s="13"/>
-      <c r="E13" s="32">
+      <c r="E13" s="31">
         <v>2967</v>
       </c>
-      <c r="F13" s="32">
+      <c r="F13" s="31">
         <v>4709.3</v>
       </c>
-      <c r="G13" s="32">
+      <c r="G13" s="31">
         <v>6528.2</v>
       </c>
-      <c r="H13" s="32">
+      <c r="H13" s="31">
         <v>8643</v>
       </c>
-      <c r="I13" s="32">
+      <c r="I13" s="31">
         <v>117.5</v>
       </c>
-      <c r="J13" s="32">
+      <c r="J13" s="31">
         <v>552.6</v>
       </c>
       <c r="K13" s="13">
         <f>J13*6.05</f>
         <v>3343.23</v>
       </c>
-      <c r="L13" s="32">
+      <c r="L13" s="31">
         <f>K13*2.7</f>
         <v>9026.7210000000014</v>
       </c>
-      <c r="M13" s="32">
+      <c r="M13" s="31">
         <f>L13*1.8</f>
         <v>16248.097800000003</v>
       </c>
-      <c r="N13" s="32">
+      <c r="N13" s="31">
         <f>M13*1.6</f>
         <v>25996.956480000008</v>
       </c>
-      <c r="O13" s="32">
+      <c r="O13" s="31">
         <f>N13*1.3</f>
         <v>33796.04342400001</v>
       </c>
-      <c r="P13" s="32">
+      <c r="P13" s="31">
         <f>O13*1.2</f>
         <v>40555.252108800014</v>
       </c>
-      <c r="Q13" s="32">
+      <c r="Q13" s="31">
         <f>P13*1.17</f>
         <v>47449.644967296015</v>
       </c>
-      <c r="R13" s="32">
+      <c r="R13" s="31">
         <f>Q13*1.15</f>
         <v>54567.091712390415</v>
       </c>
-      <c r="S13" s="32">
+      <c r="S13" s="31">
         <f>R13*1.1</f>
         <v>60023.800883629461</v>
       </c>
-      <c r="T13" s="32">
+      <c r="T13" s="31">
         <f>S13*1.07</f>
         <v>64225.466945483524</v>
       </c>
-      <c r="U13" s="30"/>
+      <c r="U13" s="29"/>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B14" s="14" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C14" s="14"/>
       <c r="D14" s="14"/>
-      <c r="E14" s="31"/>
-      <c r="F14" s="31">
+      <c r="E14" s="30"/>
+      <c r="F14" s="30">
         <f t="shared" ref="F14:J14" si="0">F13/E13-1</f>
         <v>0.58722615436467818</v>
       </c>
-      <c r="G14" s="31">
+      <c r="G14" s="30">
         <f t="shared" si="0"/>
         <v>0.38623574628925739</v>
       </c>
-      <c r="H14" s="31">
+      <c r="H14" s="30">
         <f t="shared" si="0"/>
         <v>0.32394840844336881</v>
       </c>
-      <c r="I14" s="31">
+      <c r="I14" s="30">
         <f t="shared" si="0"/>
         <v>-0.98640518338539862</v>
       </c>
-      <c r="J14" s="31">
+      <c r="J14" s="30">
         <f t="shared" si="0"/>
         <v>3.7029787234042555</v>
       </c>
-      <c r="K14" s="31">
+      <c r="K14" s="30">
         <f>K13/J13-1</f>
         <v>5.05</v>
       </c>
-      <c r="L14" s="31">
+      <c r="L14" s="30">
         <f t="shared" ref="L14:T14" si="1">L13/K13-1</f>
         <v>1.7000000000000002</v>
       </c>
-      <c r="M14" s="31">
+      <c r="M14" s="30">
         <f t="shared" si="1"/>
         <v>0.8</v>
       </c>
-      <c r="N14" s="31">
+      <c r="N14" s="30">
         <f t="shared" si="1"/>
         <v>0.60000000000000009</v>
       </c>
-      <c r="O14" s="31">
+      <c r="O14" s="30">
         <f t="shared" si="1"/>
         <v>0.30000000000000004</v>
       </c>
-      <c r="P14" s="31">
+      <c r="P14" s="30">
         <f t="shared" si="1"/>
         <v>0.19999999999999996</v>
       </c>
-      <c r="Q14" s="31">
+      <c r="Q14" s="30">
         <f t="shared" si="1"/>
         <v>0.16999999999999993</v>
       </c>
-      <c r="R14" s="31">
+      <c r="R14" s="30">
         <f t="shared" si="1"/>
         <v>0.14999999999999991</v>
       </c>
-      <c r="S14" s="31">
+      <c r="S14" s="30">
         <f t="shared" si="1"/>
         <v>0.10000000000000009</v>
       </c>
-      <c r="T14" s="31">
+      <c r="T14" s="30">
         <f t="shared" si="1"/>
         <v>7.0000000000000062E-2</v>
       </c>
-      <c r="U14" s="33"/>
+      <c r="U14" s="32"/>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B15" s="59" t="s">
-        <v>113</v>
+      <c r="B15" s="44" t="s">
+        <v>111</v>
       </c>
       <c r="E15" s="11"/>
       <c r="F15" s="11"/>
       <c r="G15" s="11"/>
       <c r="H15" s="11"/>
       <c r="I15" s="11"/>
-      <c r="J15" s="43">
+      <c r="J15" s="42">
         <f>J13*3/$R$8</f>
         <v>6.4007722007722014</v>
       </c>
-      <c r="K15" s="43">
+      <c r="K15" s="42">
         <f t="shared" ref="K15:T15" si="2">K13*3/$R$8</f>
         <v>38.724671814671815</v>
       </c>
-      <c r="L15" s="43">
+      <c r="L15" s="42">
         <f t="shared" si="2"/>
         <v>104.55661389961392</v>
       </c>
-      <c r="M15" s="43">
+      <c r="M15" s="42">
         <f t="shared" si="2"/>
         <v>188.20190501930506</v>
       </c>
-      <c r="N15" s="43">
+      <c r="N15" s="42">
         <f t="shared" si="2"/>
         <v>301.12304803088813</v>
       </c>
-      <c r="O15" s="43">
+      <c r="O15" s="42">
         <f t="shared" si="2"/>
         <v>391.45996244015458</v>
       </c>
-      <c r="P15" s="43">
+      <c r="P15" s="42">
         <f t="shared" si="2"/>
         <v>469.75195492818546</v>
       </c>
-      <c r="Q15" s="43">
+      <c r="Q15" s="42">
         <f t="shared" si="2"/>
         <v>549.60978726597705</v>
       </c>
-      <c r="R15" s="43">
+      <c r="R15" s="42">
         <f t="shared" si="2"/>
         <v>632.05125535587354</v>
       </c>
-      <c r="S15" s="43">
+      <c r="S15" s="42">
         <f t="shared" si="2"/>
         <v>695.25638089146094</v>
       </c>
-      <c r="T15" s="43">
+      <c r="T15" s="42">
         <f t="shared" si="2"/>
         <v>743.92432755386324</v>
       </c>
-      <c r="U15" s="27"/>
+      <c r="U15" s="26"/>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B16" s="41" t="s">
-        <v>111</v>
+      <c r="B16" s="40" t="s">
+        <v>109</v>
       </c>
       <c r="E16" s="11"/>
       <c r="F16" s="11"/>
       <c r="G16" s="11"/>
       <c r="H16" s="11"/>
       <c r="I16" s="11"/>
-      <c r="J16" s="43">
-        <f>PV($E$53, J63, 0, J15)*-1</f>
+      <c r="J16" s="42">
+        <f t="shared" ref="J16:T16" si="3">PV($E$53, J63, 0, J15)*-1</f>
         <v>6.4007722007722014</v>
       </c>
-      <c r="K16" s="43">
-        <f>PV($E$53, K63, 0, K15)*-1</f>
+      <c r="K16" s="42">
+        <f t="shared" si="3"/>
         <v>34.758703720197303</v>
       </c>
-      <c r="L16" s="43">
-        <f>PV($E$53, L63, 0, L15)*-1</f>
+      <c r="L16" s="42">
+        <f t="shared" si="3"/>
         <v>84.237052369206296</v>
       </c>
-      <c r="M16" s="43">
-        <f>PV($E$53, M63, 0, M15)*-1</f>
+      <c r="M16" s="42">
+        <f t="shared" si="3"/>
         <v>136.09792142946893</v>
       </c>
-      <c r="N16" s="43">
-        <f>PV($E$53, N63, 0, N15)*-1</f>
+      <c r="N16" s="42">
+        <f t="shared" si="3"/>
         <v>195.45523228359238</v>
       </c>
-      <c r="O16" s="43">
-        <f>PV($E$53, O63, 0, O15)*-1</f>
+      <c r="O16" s="42">
+        <f t="shared" si="3"/>
         <v>228.06911585016613</v>
       </c>
-      <c r="P16" s="43">
-        <f>PV($E$53, P63, 0, P15)*-1</f>
+      <c r="P16" s="42">
+        <f t="shared" si="3"/>
         <v>245.65383629853633</v>
       </c>
-      <c r="Q16" s="43">
-        <f>PV($E$53, Q63, 0, Q15)*-1</f>
+      <c r="Q16" s="42">
+        <f t="shared" si="3"/>
         <v>257.97952470091332</v>
       </c>
-      <c r="R16" s="43">
-        <f>PV($E$53, R63, 0, R15)*-1</f>
+      <c r="R16" s="42">
+        <f t="shared" si="3"/>
         <v>266.29248129077303</v>
       </c>
-      <c r="S16" s="43">
-        <f>PV($E$53, S63, 0, S15)*-1</f>
+      <c r="S16" s="42">
+        <f t="shared" si="3"/>
         <v>262.92229550296236</v>
       </c>
-      <c r="T16" s="43">
-        <f>PV($E$53, T63, 0, T15)*-1</f>
+      <c r="T16" s="42">
+        <f t="shared" si="3"/>
         <v>252.51490547362869</v>
       </c>
-      <c r="U16" s="27"/>
+      <c r="U16" s="26"/>
     </row>
     <row r="17" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="B17" s="59"/>
+      <c r="B17" s="44"/>
       <c r="E17" s="11"/>
       <c r="F17" s="11"/>
       <c r="G17" s="11"/>
@@ -1595,14 +1576,14 @@
       <c r="N17" s="11"/>
       <c r="O17" s="11"/>
       <c r="P17" s="11"/>
-      <c r="Q17" s="26"/>
-      <c r="R17" s="26"/>
+      <c r="Q17" s="25"/>
+      <c r="R17" s="25"/>
       <c r="T17" s="6"/>
-      <c r="U17" s="27"/>
+      <c r="U17" s="26"/>
     </row>
     <row r="18" spans="2:21" x14ac:dyDescent="0.3">
       <c r="B18" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E18" s="11">
         <v>220.5</v>
@@ -1626,28 +1607,28 @@
         <v>-294.60000000000002</v>
       </c>
       <c r="L18" s="11">
-        <f>L13*0.1</f>
-        <v>902.67210000000023</v>
+        <f>L13*0.04</f>
+        <v>361.06884000000008</v>
       </c>
       <c r="M18" s="11">
-        <f>M13*0.14</f>
-        <v>2274.7336920000007</v>
+        <f>M13*0.09</f>
+        <v>1462.3288020000002</v>
       </c>
       <c r="N18" s="11">
-        <f>N13*0.16</f>
-        <v>4159.5130368000009</v>
+        <f>N13*0.12</f>
+        <v>3119.6347776000007</v>
       </c>
       <c r="O18" s="11">
-        <f>O13*0.18</f>
-        <v>6083.2878163200021</v>
+        <f>O13*0.15</f>
+        <v>5069.4065136000017</v>
       </c>
       <c r="P18" s="11">
-        <f>P13*0.2</f>
-        <v>8111.0504217600028</v>
+        <f>P13*0.18</f>
+        <v>7299.9453795840027</v>
       </c>
       <c r="Q18" s="11">
-        <f>Q13*0.22</f>
-        <v>10438.921892805123</v>
+        <f>Q13*0.21</f>
+        <v>9964.4254431321624</v>
       </c>
       <c r="R18" s="11">
         <f>R13*0.23</f>
@@ -1665,101 +1646,101 @@
     </row>
     <row r="19" spans="2:21" x14ac:dyDescent="0.3">
       <c r="B19" s="14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C19" s="14"/>
       <c r="D19" s="14"/>
-      <c r="E19" s="31">
-        <f>E18/E13</f>
+      <c r="E19" s="30">
+        <f t="shared" ref="E19:T19" si="4">E18/E13</f>
         <v>7.4317492416582406E-2</v>
       </c>
-      <c r="F19" s="31">
-        <f>F18/F13</f>
+      <c r="F19" s="30">
+        <f t="shared" si="4"/>
         <v>-3.694816639415624E-2</v>
       </c>
-      <c r="G19" s="31">
-        <f>G18/G13</f>
+      <c r="G19" s="30">
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="H19" s="31">
-        <f>H18/H13</f>
+      <c r="H19" s="30">
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="I19" s="31">
-        <f>I18/I13</f>
+      <c r="I19" s="30">
+        <f t="shared" si="4"/>
         <v>-3.2885106382978719</v>
       </c>
-      <c r="J19" s="31">
-        <f>J18/J13</f>
+      <c r="J19" s="30">
+        <f t="shared" si="4"/>
         <v>-1.1791530944625408</v>
       </c>
-      <c r="K19" s="31">
-        <f>K18/K13</f>
+      <c r="K19" s="30">
+        <f t="shared" si="4"/>
         <v>-8.8118376540052584E-2</v>
       </c>
-      <c r="L19" s="31">
-        <f>L18/L13</f>
-        <v>0.1</v>
-      </c>
-      <c r="M19" s="31">
-        <f>M18/M13</f>
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="N19" s="31">
-        <f>N18/N13</f>
-        <v>0.15999999999999998</v>
-      </c>
-      <c r="O19" s="31">
-        <f>O18/O13</f>
+      <c r="L19" s="30">
+        <f t="shared" si="4"/>
+        <v>0.04</v>
+      </c>
+      <c r="M19" s="30">
+        <f t="shared" si="4"/>
+        <v>0.09</v>
+      </c>
+      <c r="N19" s="30">
+        <f t="shared" si="4"/>
+        <v>0.12</v>
+      </c>
+      <c r="O19" s="30">
+        <f t="shared" si="4"/>
+        <v>0.15</v>
+      </c>
+      <c r="P19" s="30">
+        <f t="shared" si="4"/>
         <v>0.18</v>
       </c>
-      <c r="P19" s="31">
-        <f>P18/P13</f>
-        <v>0.2</v>
-      </c>
-      <c r="Q19" s="31">
-        <f>Q18/Q13</f>
-        <v>0.22</v>
-      </c>
-      <c r="R19" s="31">
-        <f>R18/R13</f>
+      <c r="Q19" s="30">
+        <f t="shared" si="4"/>
+        <v>0.21</v>
+      </c>
+      <c r="R19" s="30">
+        <f t="shared" si="4"/>
         <v>0.23</v>
       </c>
-      <c r="S19" s="31">
-        <f>S18/S13</f>
+      <c r="S19" s="30">
+        <f t="shared" si="4"/>
         <v>0.24</v>
       </c>
-      <c r="T19" s="31">
-        <f>T18/T13</f>
+      <c r="T19" s="30">
+        <f t="shared" si="4"/>
         <v>0.25</v>
       </c>
-      <c r="U19" s="27"/>
+      <c r="U19" s="26"/>
     </row>
     <row r="20" spans="2:21" x14ac:dyDescent="0.3">
       <c r="B20" s="14"/>
       <c r="C20" s="14"/>
       <c r="D20" s="14"/>
-      <c r="E20" s="31"/>
-      <c r="F20" s="31"/>
-      <c r="G20" s="31"/>
-      <c r="H20" s="31"/>
-      <c r="I20" s="31"/>
-      <c r="J20" s="31"/>
-      <c r="K20" s="31"/>
-      <c r="L20" s="31"/>
-      <c r="M20" s="31"/>
-      <c r="N20" s="31"/>
-      <c r="O20" s="31"/>
-      <c r="P20" s="31"/>
-      <c r="Q20" s="31"/>
-      <c r="R20" s="31"/>
-      <c r="S20" s="31"/>
-      <c r="T20" s="31"/>
-      <c r="U20" s="27"/>
+      <c r="E20" s="30"/>
+      <c r="F20" s="30"/>
+      <c r="G20" s="30"/>
+      <c r="H20" s="30"/>
+      <c r="I20" s="30"/>
+      <c r="J20" s="30"/>
+      <c r="K20" s="30"/>
+      <c r="L20" s="30"/>
+      <c r="M20" s="30"/>
+      <c r="N20" s="30"/>
+      <c r="O20" s="30"/>
+      <c r="P20" s="30"/>
+      <c r="Q20" s="30"/>
+      <c r="R20" s="30"/>
+      <c r="S20" s="30"/>
+      <c r="T20" s="30"/>
+      <c r="U20" s="26"/>
     </row>
     <row r="21" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="B21" s="41" t="s">
-        <v>109</v>
+      <c r="B21" s="40" t="s">
+        <v>107</v>
       </c>
       <c r="E21" s="11"/>
       <c r="F21" s="11"/>
@@ -1777,23 +1758,23 @@
       </c>
       <c r="M21" s="11">
         <f>M18*0.1</f>
-        <v>227.47336920000009</v>
+        <v>146.23288020000004</v>
       </c>
       <c r="N21" s="11">
         <f>N18*0.12</f>
-        <v>499.14156441600011</v>
+        <v>374.35617331200007</v>
       </c>
       <c r="O21" s="11">
         <f>O18*0.14</f>
-        <v>851.66029428480033</v>
+        <v>709.71691190400031</v>
       </c>
       <c r="P21" s="11">
-        <f t="shared" ref="P21:Q21" si="3">P18*0.15</f>
-        <v>1216.6575632640004</v>
+        <f t="shared" ref="P21:Q21" si="5">P18*0.15</f>
+        <v>1094.9918069376004</v>
       </c>
       <c r="Q21" s="11">
-        <f t="shared" si="3"/>
-        <v>1565.8382839207684</v>
+        <f t="shared" si="5"/>
+        <v>1494.6638164698243</v>
       </c>
       <c r="R21" s="11">
         <f>R18*0.17</f>
@@ -1807,90 +1788,90 @@
         <f>T18*0.2</f>
         <v>3211.2733472741766</v>
       </c>
-      <c r="U21" s="27"/>
+      <c r="U21" s="26"/>
     </row>
     <row r="22" spans="2:21" x14ac:dyDescent="0.3">
       <c r="B22" s="14" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C22" s="14"/>
       <c r="D22" s="14"/>
-      <c r="E22" s="31"/>
-      <c r="F22" s="31"/>
-      <c r="G22" s="31"/>
-      <c r="H22" s="31"/>
-      <c r="I22" s="31"/>
-      <c r="J22" s="31">
+      <c r="E22" s="30"/>
+      <c r="F22" s="30"/>
+      <c r="G22" s="30"/>
+      <c r="H22" s="30"/>
+      <c r="I22" s="30"/>
+      <c r="J22" s="30">
         <f>J21/J18</f>
         <v>0</v>
       </c>
-      <c r="K22" s="31">
-        <f t="shared" ref="K22:T22" si="4">K21/K18</f>
+      <c r="K22" s="30">
+        <f t="shared" ref="K22:T22" si="6">K21/K18</f>
         <v>0</v>
       </c>
-      <c r="L22" s="31">
-        <f t="shared" si="4"/>
+      <c r="L22" s="30">
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="M22" s="31">
-        <f t="shared" si="4"/>
+      <c r="M22" s="30">
+        <f t="shared" si="6"/>
         <v>0.1</v>
       </c>
-      <c r="N22" s="31">
-        <f t="shared" si="4"/>
+      <c r="N22" s="30">
+        <f t="shared" si="6"/>
         <v>0.12</v>
       </c>
-      <c r="O22" s="31">
-        <f t="shared" si="4"/>
+      <c r="O22" s="30">
+        <f t="shared" si="6"/>
         <v>0.14000000000000001</v>
       </c>
-      <c r="P22" s="31">
-        <f t="shared" si="4"/>
+      <c r="P22" s="30">
+        <f t="shared" si="6"/>
         <v>0.15</v>
       </c>
-      <c r="Q22" s="31">
-        <f t="shared" si="4"/>
+      <c r="Q22" s="30">
+        <f t="shared" si="6"/>
         <v>0.15</v>
       </c>
-      <c r="R22" s="31">
-        <f t="shared" si="4"/>
+      <c r="R22" s="30">
+        <f t="shared" si="6"/>
         <v>0.17</v>
       </c>
-      <c r="S22" s="31">
-        <f t="shared" si="4"/>
+      <c r="S22" s="30">
+        <f t="shared" si="6"/>
         <v>0.18</v>
       </c>
-      <c r="T22" s="31">
-        <f t="shared" si="4"/>
+      <c r="T22" s="30">
+        <f t="shared" si="6"/>
         <v>0.2</v>
       </c>
-      <c r="U22" s="27"/>
+      <c r="U22" s="26"/>
     </row>
     <row r="23" spans="2:21" x14ac:dyDescent="0.3">
       <c r="B23" s="14"/>
       <c r="C23" s="14"/>
       <c r="D23" s="14"/>
-      <c r="E23" s="31"/>
-      <c r="F23" s="31"/>
-      <c r="G23" s="31"/>
-      <c r="H23" s="31"/>
-      <c r="I23" s="31"/>
-      <c r="J23" s="31"/>
-      <c r="K23" s="31"/>
-      <c r="L23" s="31"/>
-      <c r="M23" s="31"/>
-      <c r="N23" s="31"/>
-      <c r="O23" s="31"/>
-      <c r="P23" s="31"/>
-      <c r="Q23" s="31"/>
-      <c r="R23" s="31"/>
-      <c r="S23" s="31"/>
-      <c r="T23" s="31"/>
-      <c r="U23" s="27"/>
+      <c r="E23" s="30"/>
+      <c r="F23" s="30"/>
+      <c r="G23" s="30"/>
+      <c r="H23" s="30"/>
+      <c r="I23" s="30"/>
+      <c r="J23" s="30"/>
+      <c r="K23" s="30"/>
+      <c r="L23" s="30"/>
+      <c r="M23" s="30"/>
+      <c r="N23" s="30"/>
+      <c r="O23" s="30"/>
+      <c r="P23" s="30"/>
+      <c r="Q23" s="30"/>
+      <c r="R23" s="30"/>
+      <c r="S23" s="30"/>
+      <c r="T23" s="30"/>
+      <c r="U23" s="26"/>
     </row>
     <row r="24" spans="2:21" x14ac:dyDescent="0.3">
       <c r="B24" s="1" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="E24" s="11"/>
       <c r="F24" s="11"/>
@@ -1902,54 +1883,54 @@
         <v>-651.6</v>
       </c>
       <c r="K24" s="11">
-        <f t="shared" ref="K24:T24" si="5">K18-K21</f>
+        <f t="shared" ref="K24:T24" si="7">K18-K21</f>
         <v>-294.60000000000002</v>
       </c>
       <c r="L24" s="11">
-        <f t="shared" si="5"/>
-        <v>902.67210000000023</v>
+        <f t="shared" si="7"/>
+        <v>361.06884000000008</v>
       </c>
       <c r="M24" s="11">
-        <f t="shared" si="5"/>
-        <v>2047.2603228000007</v>
+        <f t="shared" si="7"/>
+        <v>1316.0959218000003</v>
       </c>
       <c r="N24" s="11">
-        <f t="shared" si="5"/>
-        <v>3660.3714723840008</v>
+        <f t="shared" si="7"/>
+        <v>2745.2786042880007</v>
       </c>
       <c r="O24" s="11">
-        <f t="shared" si="5"/>
-        <v>5231.6275220352018</v>
+        <f t="shared" si="7"/>
+        <v>4359.6896016960018</v>
       </c>
       <c r="P24" s="11">
-        <f t="shared" si="5"/>
-        <v>6894.3928584960022</v>
+        <f t="shared" si="7"/>
+        <v>6204.9535726464019</v>
       </c>
       <c r="Q24" s="11">
-        <f t="shared" si="5"/>
-        <v>8873.0836088843553</v>
+        <f t="shared" si="7"/>
+        <v>8469.7616266623372</v>
       </c>
       <c r="R24" s="11">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>10416.857807895331</v>
       </c>
       <c r="S24" s="11">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>11812.684013898277</v>
       </c>
       <c r="T24" s="11">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>12845.093389096704</v>
       </c>
-      <c r="U24" s="27"/>
+      <c r="U24" s="26"/>
     </row>
     <row r="25" spans="2:21" x14ac:dyDescent="0.3">
       <c r="P25" s="11"/>
       <c r="Q25" s="11"/>
     </row>
     <row r="26" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="B26" s="41" t="s">
-        <v>40</v>
+      <c r="B26" s="40" t="s">
+        <v>39</v>
       </c>
       <c r="E26" s="11">
         <v>240.3</v>
@@ -1975,188 +1956,188 @@
         <v>2068.8876</v>
       </c>
       <c r="L26" s="11">
-        <f>L30*0.32</f>
-        <v>4965.3302400000002</v>
+        <f>L30*0.34</f>
+        <v>5275.6633800000009</v>
       </c>
       <c r="M26" s="11">
-        <f>M30*0.35</f>
-        <v>6788.5374375000001</v>
+        <f>M30*0.4</f>
+        <v>7758.3285000000005</v>
       </c>
       <c r="N26" s="11">
-        <f>N13*0.4</f>
+        <f t="shared" ref="N26:T26" si="8">N13*0.4</f>
         <v>10398.782592000003</v>
       </c>
       <c r="O26" s="11">
-        <f>O13*0.4</f>
+        <f t="shared" si="8"/>
         <v>13518.417369600005</v>
       </c>
       <c r="P26" s="11">
-        <f>P13*0.4</f>
+        <f t="shared" si="8"/>
         <v>16222.100843520006</v>
       </c>
       <c r="Q26" s="11">
-        <f>Q13*0.4</f>
+        <f t="shared" si="8"/>
         <v>18979.857986918407</v>
       </c>
       <c r="R26" s="11">
-        <f>R13*0.4</f>
+        <f t="shared" si="8"/>
         <v>21826.836684956168</v>
       </c>
       <c r="S26" s="11">
-        <f>S13*0.4</f>
+        <f t="shared" si="8"/>
         <v>24009.520353451786</v>
       </c>
       <c r="T26" s="11">
-        <f>T13*0.4</f>
+        <f t="shared" si="8"/>
         <v>25690.186778193412</v>
       </c>
     </row>
     <row r="27" spans="2:21" x14ac:dyDescent="0.3">
       <c r="B27" s="14" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C27" s="14"/>
       <c r="D27" s="14"/>
-      <c r="E27" s="31">
+      <c r="E27" s="30">
         <f>E26/E30</f>
         <v>0.72598187311178253</v>
       </c>
-      <c r="F27" s="31">
+      <c r="F27" s="30">
         <f>F26/F30</f>
         <v>0.53864406779661023</v>
       </c>
-      <c r="G27" s="31"/>
-      <c r="H27" s="31"/>
-      <c r="I27" s="31">
-        <f t="shared" ref="I27:T27" si="6">I26/I30</f>
+      <c r="G27" s="30"/>
+      <c r="H27" s="30"/>
+      <c r="I27" s="30">
+        <f t="shared" ref="I27:T27" si="9">I26/I30</f>
         <v>9.566831683168317E-2</v>
       </c>
-      <c r="J27" s="31">
-        <f t="shared" si="6"/>
+      <c r="J27" s="30">
+        <f t="shared" si="9"/>
         <v>0.105</v>
       </c>
-      <c r="K27" s="31">
-        <f t="shared" si="6"/>
+      <c r="K27" s="30">
+        <f t="shared" si="9"/>
         <v>0.18</v>
       </c>
-      <c r="L27" s="31">
-        <f t="shared" si="6"/>
-        <v>0.32</v>
-      </c>
-      <c r="M27" s="31">
-        <f t="shared" si="6"/>
-        <v>0.35</v>
-      </c>
-      <c r="N27" s="31">
-        <f t="shared" si="6"/>
+      <c r="L27" s="30">
+        <f t="shared" si="9"/>
+        <v>0.34</v>
+      </c>
+      <c r="M27" s="30">
+        <f t="shared" si="9"/>
+        <v>0.4</v>
+      </c>
+      <c r="N27" s="30">
+        <f t="shared" si="9"/>
         <v>0.48739564043981909</v>
       </c>
-      <c r="O27" s="31">
-        <f t="shared" si="6"/>
+      <c r="O27" s="30">
+        <f t="shared" si="9"/>
         <v>0.57601302961069523</v>
       </c>
-      <c r="P27" s="31">
-        <f t="shared" si="6"/>
+      <c r="P27" s="30">
+        <f t="shared" si="9"/>
         <v>0.64001447734521688</v>
       </c>
-      <c r="Q27" s="31">
-        <f t="shared" si="6"/>
+      <c r="Q27" s="30">
+        <f t="shared" si="9"/>
         <v>0.73413425342539584</v>
       </c>
-      <c r="R27" s="31">
-        <f t="shared" si="6"/>
+      <c r="R27" s="30">
+        <f t="shared" si="9"/>
         <v>0.82770038376392674</v>
       </c>
-      <c r="S27" s="31">
-        <f t="shared" si="6"/>
+      <c r="S27" s="30">
+        <f t="shared" si="9"/>
         <v>0.8926180609218819</v>
       </c>
-      <c r="T27" s="31">
-        <f t="shared" si="6"/>
+      <c r="T27" s="30">
+        <f t="shared" si="9"/>
         <v>0.93637384822197423</v>
       </c>
     </row>
     <row r="28" spans="2:21" x14ac:dyDescent="0.3">
       <c r="B28" s="14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C28" s="14"/>
       <c r="D28" s="14"/>
-      <c r="E28" s="31">
-        <f>E26/E13</f>
+      <c r="E28" s="30">
+        <f t="shared" ref="E28:T28" si="10">E26/E13</f>
         <v>8.0990899898887775E-2</v>
       </c>
-      <c r="F28" s="31">
-        <f>F26/F13</f>
+      <c r="F28" s="30">
+        <f t="shared" si="10"/>
         <v>6.748349011530376E-2</v>
       </c>
-      <c r="G28" s="31">
-        <f>G26/G13</f>
+      <c r="G28" s="30">
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="H28" s="31">
-        <f>H26/H13</f>
+      <c r="H28" s="30">
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="I28" s="31">
-        <f>I26/I13</f>
+      <c r="I28" s="30">
+        <f t="shared" si="10"/>
         <v>0.65787234042553189</v>
       </c>
-      <c r="J28" s="31">
-        <f>J26/J13</f>
+      <c r="J28" s="30">
+        <f t="shared" si="10"/>
         <v>0.83998099891422362</v>
       </c>
-      <c r="K28" s="31">
-        <f>K26/K13</f>
+      <c r="K28" s="30">
+        <f t="shared" si="10"/>
         <v>0.61882897676797588</v>
       </c>
-      <c r="L28" s="31">
-        <f>L26/L13</f>
-        <v>0.55007020157153408</v>
-      </c>
-      <c r="M28" s="31">
-        <f>M26/M13</f>
-        <v>0.41780505761726761</v>
-      </c>
-      <c r="N28" s="31">
-        <f>N26/N13</f>
+      <c r="L28" s="30">
+        <f t="shared" si="10"/>
+        <v>0.58444958916975498</v>
+      </c>
+      <c r="M28" s="30">
+        <f t="shared" si="10"/>
+        <v>0.47749149441973443</v>
+      </c>
+      <c r="N28" s="30">
+        <f t="shared" si="10"/>
         <v>0.4</v>
       </c>
-      <c r="O28" s="31">
-        <f>O26/O13</f>
+      <c r="O28" s="30">
+        <f t="shared" si="10"/>
         <v>0.4</v>
       </c>
-      <c r="P28" s="31">
-        <f>P26/P13</f>
+      <c r="P28" s="30">
+        <f t="shared" si="10"/>
         <v>0.4</v>
       </c>
-      <c r="Q28" s="31">
-        <f>Q26/Q13</f>
+      <c r="Q28" s="30">
+        <f t="shared" si="10"/>
         <v>0.4</v>
       </c>
-      <c r="R28" s="31">
-        <f>R26/R13</f>
+      <c r="R28" s="30">
+        <f t="shared" si="10"/>
         <v>0.4</v>
       </c>
-      <c r="S28" s="31">
-        <f>S26/S13</f>
+      <c r="S28" s="30">
+        <f t="shared" si="10"/>
         <v>0.4</v>
       </c>
-      <c r="T28" s="31">
-        <f>T26/T13</f>
+      <c r="T28" s="30">
+        <f t="shared" si="10"/>
         <v>0.4</v>
       </c>
     </row>
     <row r="29" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="P29" s="31"/>
-      <c r="Q29" s="31"/>
-      <c r="R29" s="31"/>
-      <c r="S29" s="31"/>
-      <c r="T29" s="31"/>
+      <c r="P29" s="30"/>
+      <c r="Q29" s="30"/>
+      <c r="R29" s="30"/>
+      <c r="S29" s="30"/>
+      <c r="T29" s="30"/>
     </row>
     <row r="30" spans="2:21" x14ac:dyDescent="0.3">
       <c r="B30" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E30" s="11">
         <v>331</v>
@@ -2205,148 +2186,148 @@
         <v>25853.388393690006</v>
       </c>
       <c r="R30" s="11">
-        <f t="shared" ref="R30:T30" si="7">Q30*1.02</f>
+        <f t="shared" ref="R30:T30" si="11">Q30*1.02</f>
         <v>26370.456161563805</v>
       </c>
       <c r="S30" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>26897.86528479508</v>
       </c>
       <c r="T30" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="11"/>
         <v>27435.822590490981</v>
       </c>
     </row>
     <row r="31" spans="2:21" x14ac:dyDescent="0.3">
       <c r="B31" s="14" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C31" s="14"/>
       <c r="D31" s="14"/>
-      <c r="E31" s="31"/>
-      <c r="F31" s="31">
-        <f t="shared" ref="F31" si="8">F30/E30-1</f>
+      <c r="E31" s="30"/>
+      <c r="F31" s="30">
+        <f t="shared" ref="F31" si="12">F30/E30-1</f>
         <v>0.78247734138972813</v>
       </c>
-      <c r="G31" s="31">
-        <f t="shared" ref="G31" si="9">G30/F30-1</f>
+      <c r="G31" s="30">
+        <f t="shared" ref="G31" si="13">G30/F30-1</f>
         <v>-1</v>
       </c>
-      <c r="H31" s="31"/>
-      <c r="I31" s="31"/>
-      <c r="J31" s="31">
-        <f t="shared" ref="J31" si="10">J30/I30-1</f>
+      <c r="H31" s="30"/>
+      <c r="I31" s="30"/>
+      <c r="J31" s="30">
+        <f t="shared" ref="J31" si="14">J30/I30-1</f>
         <v>4.4711633663366337</v>
       </c>
-      <c r="K31" s="31">
-        <f t="shared" ref="K31" si="11">K30/J30-1</f>
+      <c r="K31" s="30">
+        <f t="shared" ref="K31" si="15">K30/J30-1</f>
         <v>1.6</v>
       </c>
-      <c r="L31" s="31">
-        <f t="shared" ref="L31" si="12">L30/K30-1</f>
+      <c r="L31" s="30">
+        <f t="shared" ref="L31" si="16">L30/K30-1</f>
         <v>0.35000000000000009</v>
       </c>
-      <c r="M31" s="31">
-        <f t="shared" ref="M31" si="13">M30/L30-1</f>
+      <c r="M31" s="30">
+        <f t="shared" ref="M31" si="17">M30/L30-1</f>
         <v>0.25</v>
       </c>
-      <c r="N31" s="31">
-        <f t="shared" ref="N31" si="14">N30/M30-1</f>
+      <c r="N31" s="30">
+        <f t="shared" ref="N31" si="18">N30/M30-1</f>
         <v>0.10000000000000009</v>
       </c>
-      <c r="O31" s="31">
-        <f t="shared" ref="O31" si="15">O30/N30-1</f>
+      <c r="O31" s="30">
+        <f t="shared" ref="O31" si="19">O30/N30-1</f>
         <v>0.10000000000000009</v>
       </c>
-      <c r="P31" s="31">
-        <f t="shared" ref="P31" si="16">P30/O30-1</f>
+      <c r="P31" s="30">
+        <f t="shared" ref="P31" si="20">P30/O30-1</f>
         <v>8.0000000000000071E-2</v>
       </c>
-      <c r="Q31" s="31">
-        <f t="shared" ref="Q31" si="17">Q30/P30-1</f>
+      <c r="Q31" s="30">
+        <f t="shared" ref="Q31" si="21">Q30/P30-1</f>
         <v>2.0000000000000018E-2</v>
       </c>
-      <c r="R31" s="31">
-        <f t="shared" ref="R31" si="18">R30/Q30-1</f>
+      <c r="R31" s="30">
+        <f t="shared" ref="R31" si="22">R30/Q30-1</f>
         <v>2.0000000000000018E-2</v>
       </c>
-      <c r="S31" s="31">
-        <f t="shared" ref="S31" si="19">S30/R30-1</f>
+      <c r="S31" s="30">
+        <f t="shared" ref="S31" si="23">S30/R30-1</f>
         <v>2.0000000000000018E-2</v>
       </c>
-      <c r="T31" s="31">
-        <f t="shared" ref="T31" si="20">T30/S30-1</f>
+      <c r="T31" s="30">
+        <f t="shared" ref="T31" si="24">T30/S30-1</f>
         <v>2.0000000000000018E-2</v>
       </c>
     </row>
     <row r="32" spans="2:21" x14ac:dyDescent="0.3">
       <c r="B32" s="14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C32" s="14"/>
       <c r="D32" s="14"/>
-      <c r="E32" s="31">
-        <f>E30/E13</f>
+      <c r="E32" s="30">
+        <f t="shared" ref="E32:T32" si="25">E30/E13</f>
         <v>0.11156049882035726</v>
       </c>
-      <c r="F32" s="31">
-        <f>F30/F13</f>
+      <c r="F32" s="30">
+        <f t="shared" si="25"/>
         <v>0.1252840124859321</v>
       </c>
-      <c r="G32" s="31">
-        <f>G30/G13</f>
+      <c r="G32" s="30">
+        <f t="shared" si="25"/>
         <v>0</v>
       </c>
-      <c r="H32" s="31">
-        <f>H30/H13</f>
+      <c r="H32" s="30">
+        <f t="shared" si="25"/>
         <v>0</v>
       </c>
-      <c r="I32" s="31">
-        <f>I30/I13</f>
+      <c r="I32" s="30">
+        <f t="shared" si="25"/>
         <v>6.8765957446808512</v>
       </c>
-      <c r="J32" s="31">
-        <f>J30/J13</f>
+      <c r="J32" s="30">
+        <f t="shared" si="25"/>
         <v>7.9998190372783204</v>
       </c>
-      <c r="K32" s="31">
-        <f>K30/K13</f>
+      <c r="K32" s="30">
+        <f t="shared" si="25"/>
         <v>3.4379387598220883</v>
       </c>
-      <c r="L32" s="31">
-        <f>L30/L13</f>
+      <c r="L32" s="30">
+        <f t="shared" si="25"/>
         <v>1.7189693799110439</v>
       </c>
-      <c r="M32" s="31">
-        <f>M30/M13</f>
+      <c r="M32" s="30">
+        <f t="shared" si="25"/>
         <v>1.193728736049336</v>
       </c>
-      <c r="N32" s="31">
-        <f>N30/N13</f>
+      <c r="N32" s="30">
+        <f t="shared" si="25"/>
         <v>0.82068850603391841</v>
       </c>
-      <c r="O32" s="31">
-        <f>O30/O13</f>
+      <c r="O32" s="30">
+        <f t="shared" si="25"/>
         <v>0.6944287358748541</v>
       </c>
-      <c r="P32" s="31">
-        <f>P30/P13</f>
+      <c r="P32" s="30">
+        <f t="shared" si="25"/>
         <v>0.62498586228736874</v>
       </c>
-      <c r="Q32" s="31">
-        <f>Q30/Q13</f>
+      <c r="Q32" s="30">
+        <f t="shared" si="25"/>
         <v>0.54485946968642407</v>
       </c>
-      <c r="R32" s="31">
-        <f>R30/R13</f>
+      <c r="R32" s="30">
+        <f t="shared" si="25"/>
         <v>0.48326666006969782</v>
       </c>
-      <c r="S32" s="31">
-        <f>S30/S13</f>
+      <c r="S32" s="30">
+        <f t="shared" si="25"/>
         <v>0.44811999388281065</v>
       </c>
-      <c r="T32" s="31">
-        <f>T30/T13</f>
+      <c r="T32" s="30">
+        <f t="shared" si="25"/>
         <v>0.42717980725277277</v>
       </c>
     </row>
@@ -2354,26 +2335,26 @@
       <c r="B33" s="14"/>
       <c r="C33" s="14"/>
       <c r="D33" s="14"/>
-      <c r="E33" s="31"/>
-      <c r="F33" s="31"/>
-      <c r="G33" s="31"/>
-      <c r="H33" s="31"/>
-      <c r="I33" s="31"/>
-      <c r="J33" s="31"/>
-      <c r="K33" s="31"/>
-      <c r="L33" s="31"/>
-      <c r="M33" s="31"/>
-      <c r="N33" s="31"/>
-      <c r="O33" s="31"/>
-      <c r="P33" s="31"/>
-      <c r="Q33" s="31"/>
-      <c r="R33" s="31"/>
-      <c r="S33" s="31"/>
-      <c r="T33" s="31"/>
+      <c r="E33" s="30"/>
+      <c r="F33" s="30"/>
+      <c r="G33" s="30"/>
+      <c r="H33" s="30"/>
+      <c r="I33" s="30"/>
+      <c r="J33" s="30"/>
+      <c r="K33" s="30"/>
+      <c r="L33" s="30"/>
+      <c r="M33" s="30"/>
+      <c r="N33" s="30"/>
+      <c r="O33" s="30"/>
+      <c r="P33" s="30"/>
+      <c r="Q33" s="30"/>
+      <c r="R33" s="30"/>
+      <c r="S33" s="30"/>
+      <c r="T33" s="30"/>
     </row>
     <row r="34" spans="2:21" x14ac:dyDescent="0.3">
       <c r="B34" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E34" s="11"/>
       <c r="F34" s="11"/>
@@ -2381,212 +2362,212 @@
       <c r="H34" s="11"/>
       <c r="I34" s="11"/>
       <c r="J34" s="11">
-        <f>J24+24</f>
-        <v>-627.6</v>
+        <f>J24-J26</f>
+        <v>-1115.7735</v>
       </c>
       <c r="K34" s="11">
-        <f t="shared" ref="K34:T34" si="21">K24+24</f>
-        <v>-270.60000000000002</v>
+        <f t="shared" ref="K34:T34" si="26">K24</f>
+        <v>-294.60000000000002</v>
       </c>
       <c r="L34" s="11">
-        <f t="shared" si="21"/>
-        <v>926.67210000000023</v>
+        <f t="shared" si="26"/>
+        <v>361.06884000000008</v>
       </c>
       <c r="M34" s="11">
-        <f t="shared" si="21"/>
-        <v>2071.2603228000007</v>
+        <f t="shared" si="26"/>
+        <v>1316.0959218000003</v>
       </c>
       <c r="N34" s="11">
-        <f t="shared" si="21"/>
-        <v>3684.3714723840008</v>
+        <f t="shared" si="26"/>
+        <v>2745.2786042880007</v>
       </c>
       <c r="O34" s="11">
-        <f t="shared" si="21"/>
-        <v>5255.6275220352018</v>
+        <f t="shared" si="26"/>
+        <v>4359.6896016960018</v>
       </c>
       <c r="P34" s="11">
-        <f t="shared" si="21"/>
-        <v>6918.3928584960022</v>
+        <f t="shared" si="26"/>
+        <v>6204.9535726464019</v>
       </c>
       <c r="Q34" s="11">
-        <f t="shared" si="21"/>
-        <v>8897.0836088843553</v>
+        <f t="shared" si="26"/>
+        <v>8469.7616266623372</v>
       </c>
       <c r="R34" s="11">
-        <f t="shared" si="21"/>
-        <v>10440.857807895331</v>
+        <f t="shared" si="26"/>
+        <v>10416.857807895331</v>
       </c>
       <c r="S34" s="11">
-        <f t="shared" si="21"/>
-        <v>11836.684013898277</v>
+        <f t="shared" si="26"/>
+        <v>11812.684013898277</v>
       </c>
       <c r="T34" s="11">
-        <f t="shared" si="21"/>
-        <v>12869.093389096704</v>
+        <f t="shared" si="26"/>
+        <v>12845.093389096704</v>
       </c>
     </row>
     <row r="35" spans="2:21" x14ac:dyDescent="0.3">
       <c r="B35" s="14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C35" s="14"/>
       <c r="D35" s="14"/>
-      <c r="E35" s="31"/>
-      <c r="F35" s="31"/>
-      <c r="G35" s="31"/>
-      <c r="H35" s="31"/>
-      <c r="I35" s="31"/>
-      <c r="J35" s="31">
-        <f>J34/J13</f>
-        <v>-1.1357220412595006</v>
-      </c>
-      <c r="K35" s="31">
-        <f>K34/K13</f>
-        <v>-8.0939690060211233E-2</v>
-      </c>
-      <c r="L35" s="31">
-        <f>L34/L13</f>
-        <v>0.10265877277031162</v>
-      </c>
-      <c r="M35" s="31">
-        <f>M34/M13</f>
-        <v>0.12747709598350648</v>
-      </c>
-      <c r="N35" s="31">
-        <f>N34/N13</f>
-        <v>0.14172318498969153</v>
-      </c>
-      <c r="O35" s="31">
-        <f>O34/O13</f>
-        <v>0.15551014229976273</v>
-      </c>
-      <c r="P35" s="31">
-        <f>P34/P13</f>
-        <v>0.17059178524980226</v>
-      </c>
-      <c r="Q35" s="31">
-        <f>Q34/Q13</f>
-        <v>0.18750579935880538</v>
-      </c>
-      <c r="R35" s="31">
-        <f>R34/R13</f>
-        <v>0.19133982552939596</v>
-      </c>
-      <c r="S35" s="31">
-        <f>S34/S13</f>
-        <v>0.19719984139035995</v>
-      </c>
-      <c r="T35" s="31">
-        <f>T34/T13</f>
-        <v>0.20037368354239249</v>
+      <c r="E35" s="30"/>
+      <c r="F35" s="30"/>
+      <c r="G35" s="30"/>
+      <c r="H35" s="30"/>
+      <c r="I35" s="30"/>
+      <c r="J35" s="30">
+        <f t="shared" ref="J35:T35" si="27">J34/J13</f>
+        <v>-2.0191340933767643</v>
+      </c>
+      <c r="K35" s="30">
+        <f t="shared" si="27"/>
+        <v>-8.8118376540052584E-2</v>
+      </c>
+      <c r="L35" s="30">
+        <f t="shared" si="27"/>
+        <v>0.04</v>
+      </c>
+      <c r="M35" s="30">
+        <f t="shared" si="27"/>
+        <v>8.1000000000000003E-2</v>
+      </c>
+      <c r="N35" s="30">
+        <f t="shared" si="27"/>
+        <v>0.1056</v>
+      </c>
+      <c r="O35" s="30">
+        <f t="shared" si="27"/>
+        <v>0.129</v>
+      </c>
+      <c r="P35" s="30">
+        <f t="shared" si="27"/>
+        <v>0.153</v>
+      </c>
+      <c r="Q35" s="30">
+        <f t="shared" si="27"/>
+        <v>0.17849999999999996</v>
+      </c>
+      <c r="R35" s="30">
+        <f t="shared" si="27"/>
+        <v>0.19090000000000001</v>
+      </c>
+      <c r="S35" s="30">
+        <f t="shared" si="27"/>
+        <v>0.19679999999999997</v>
+      </c>
+      <c r="T35" s="30">
+        <f t="shared" si="27"/>
+        <v>0.19999999999999998</v>
       </c>
     </row>
     <row r="36" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="B36" s="41" t="s">
-        <v>110</v>
+      <c r="B36" s="40" t="s">
+        <v>108</v>
       </c>
       <c r="E36" s="11"/>
       <c r="F36" s="11"/>
       <c r="G36" s="11"/>
       <c r="H36" s="11"/>
       <c r="I36" s="11"/>
-      <c r="J36" s="43">
+      <c r="J36" s="42">
         <f>J34*18/$R$8</f>
-        <v>-43.61698841698842</v>
-      </c>
-      <c r="K36" s="43">
-        <f t="shared" ref="K36:T36" si="22">K34*18/$R$8</f>
-        <v>-18.806177606177606</v>
-      </c>
-      <c r="L36" s="43">
-        <f t="shared" si="22"/>
-        <v>64.401922007722021</v>
-      </c>
-      <c r="M36" s="43">
-        <f t="shared" si="22"/>
-        <v>143.94859386254831</v>
-      </c>
-      <c r="N36" s="43">
-        <f t="shared" si="22"/>
-        <v>256.0567046444479</v>
-      </c>
-      <c r="O36" s="43">
-        <f t="shared" si="22"/>
-        <v>365.25596678236923</v>
-      </c>
-      <c r="P36" s="43">
-        <f t="shared" si="22"/>
-        <v>480.81494769470282</v>
-      </c>
-      <c r="Q36" s="43">
-        <f t="shared" si="22"/>
-        <v>618.33013498037985</v>
-      </c>
-      <c r="R36" s="43">
-        <f t="shared" si="22"/>
-        <v>725.61946155257124</v>
-      </c>
-      <c r="S36" s="43">
-        <f t="shared" si="22"/>
-        <v>822.62668822459068</v>
-      </c>
-      <c r="T36" s="43">
-        <f t="shared" si="22"/>
-        <v>894.37714673258949</v>
+        <v>-77.544104247104244</v>
+      </c>
+      <c r="K36" s="42">
+        <f t="shared" ref="K36:T36" si="28">K34*18/$R$8</f>
+        <v>-20.474131274131274</v>
+      </c>
+      <c r="L36" s="42">
+        <f t="shared" si="28"/>
+        <v>25.09358733590734</v>
+      </c>
+      <c r="M36" s="42">
+        <f t="shared" si="28"/>
+        <v>91.466125839382258</v>
+      </c>
+      <c r="N36" s="42">
+        <f t="shared" si="28"/>
+        <v>190.79156323237069</v>
+      </c>
+      <c r="O36" s="42">
+        <f t="shared" si="28"/>
+        <v>302.99001092867968</v>
+      </c>
+      <c r="P36" s="42">
+        <f t="shared" si="28"/>
+        <v>431.23229462407426</v>
+      </c>
+      <c r="Q36" s="42">
+        <f t="shared" si="28"/>
+        <v>588.63208216186126</v>
+      </c>
+      <c r="R36" s="42">
+        <f t="shared" si="28"/>
+        <v>723.95150788461751</v>
+      </c>
+      <c r="S36" s="42">
+        <f t="shared" si="28"/>
+        <v>820.95873455663707</v>
+      </c>
+      <c r="T36" s="42">
+        <f t="shared" si="28"/>
+        <v>892.70919306463577</v>
       </c>
     </row>
     <row r="37" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="B37" s="41" t="s">
-        <v>111</v>
+      <c r="B37" s="40" t="s">
+        <v>109</v>
       </c>
       <c r="E37" s="11"/>
       <c r="F37" s="11"/>
       <c r="G37" s="11"/>
       <c r="H37" s="11"/>
       <c r="I37" s="11"/>
-      <c r="J37" s="43">
-        <f>PV($E$53, J63, 0, J36)*-1</f>
-        <v>-43.61698841698842</v>
-      </c>
-      <c r="K37" s="43">
-        <f>PV($E$53, K63, 0, K36)*-1</f>
-        <v>-16.880152236044882</v>
-      </c>
-      <c r="L37" s="43">
-        <f>PV($E$53, L63, 0, L36)*-1</f>
-        <v>51.886034508067127</v>
-      </c>
-      <c r="M37" s="43">
-        <f>PV($E$53, M63, 0, M36)*-1</f>
-        <v>104.09620675932078</v>
-      </c>
-      <c r="N37" s="43">
-        <f>PV($E$53, N63, 0, N36)*-1</f>
-        <v>166.2032282527841</v>
-      </c>
-      <c r="O37" s="43">
-        <f>PV($E$53, O63, 0, O36)*-1</f>
-        <v>212.80236396024239</v>
-      </c>
-      <c r="P37" s="43">
-        <f>PV($E$53, P63, 0, P36)*-1</f>
-        <v>251.43915892577994</v>
-      </c>
-      <c r="Q37" s="43">
-        <f>PV($E$53, Q63, 0, Q36)*-1</f>
-        <v>290.2359419834965</v>
-      </c>
-      <c r="R37" s="43">
-        <f>PV($E$53, R63, 0, R36)*-1</f>
-        <v>305.71414145979873</v>
-      </c>
-      <c r="S37" s="43">
-        <f>PV($E$53, S63, 0, S36)*-1</f>
-        <v>311.0894098270411</v>
-      </c>
-      <c r="T37" s="43">
-        <f>PV($E$53, T63, 0, T36)*-1</f>
-        <v>303.58405055466017</v>
+      <c r="J37" s="42">
+        <f t="shared" ref="J37:T37" si="29">PV($E$53, J63, 0, J36)*-1</f>
+        <v>-77.544104247104244</v>
+      </c>
+      <c r="K37" s="42">
+        <f t="shared" si="29"/>
+        <v>-18.377283254762833</v>
+      </c>
+      <c r="L37" s="42">
+        <f t="shared" si="29"/>
+        <v>20.216892568609509</v>
+      </c>
+      <c r="M37" s="42">
+        <f t="shared" si="29"/>
+        <v>66.143589814721892</v>
+      </c>
+      <c r="N37" s="42">
+        <f t="shared" si="29"/>
+        <v>123.84043517488412</v>
+      </c>
+      <c r="O37" s="42">
+        <f t="shared" si="29"/>
+        <v>176.52549566802858</v>
+      </c>
+      <c r="P37" s="42">
+        <f t="shared" si="29"/>
+        <v>225.51022172205637</v>
+      </c>
+      <c r="Q37" s="42">
+        <f t="shared" si="29"/>
+        <v>276.2960709546781</v>
+      </c>
+      <c r="R37" s="42">
+        <f t="shared" si="29"/>
+        <v>305.01140807045141</v>
+      </c>
+      <c r="S37" s="42">
+        <f t="shared" si="29"/>
+        <v>310.45864652989792</v>
+      </c>
+      <c r="T37" s="42">
+        <f t="shared" si="29"/>
+        <v>303.01788656835436</v>
       </c>
     </row>
     <row r="38" spans="2:21" x14ac:dyDescent="0.3">
@@ -2594,7 +2575,7 @@
     </row>
     <row r="39" spans="2:21" x14ac:dyDescent="0.3">
       <c r="B39" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E39" s="11">
         <v>-93.1</v>
@@ -2612,217 +2593,217 @@
         <v>-1115</v>
       </c>
       <c r="J39" s="11">
-        <f>J24+J26-J30</f>
+        <f t="shared" ref="J39:T39" si="30">J24+J26-J30</f>
         <v>-4608.1265000000003</v>
       </c>
       <c r="K39" s="11">
-        <f>K24+K26-K30</f>
+        <f t="shared" si="30"/>
         <v>-9719.5324000000001</v>
       </c>
       <c r="L39" s="11">
-        <f>L24+L26-L30</f>
-        <v>-9648.6546600000001</v>
+        <f t="shared" si="30"/>
+        <v>-9879.9247800000012</v>
       </c>
       <c r="M39" s="11">
-        <f>M24+M26-M30</f>
-        <v>-10560.023489700001</v>
+        <f t="shared" si="30"/>
+        <v>-10321.396828200001</v>
       </c>
       <c r="N39" s="11">
-        <f>N24+N26-N30</f>
-        <v>-7276.2493106159982</v>
+        <f t="shared" si="30"/>
+        <v>-8191.3421787119987</v>
       </c>
       <c r="O39" s="11">
-        <f>O24+O26-O30</f>
-        <v>-4718.898820864797</v>
+        <f t="shared" si="30"/>
+        <v>-5590.8367412039952</v>
       </c>
       <c r="P39" s="11">
-        <f>P24+P26-P30</f>
-        <v>-2229.9655074839975</v>
+        <f t="shared" si="30"/>
+        <v>-2919.4047933335969</v>
       </c>
       <c r="Q39" s="11">
-        <f>Q24+Q26-Q30</f>
-        <v>1999.5532021127547</v>
+        <f t="shared" si="30"/>
+        <v>1596.2312198907384</v>
       </c>
       <c r="R39" s="11">
-        <f>R24+R26-R30</f>
+        <f t="shared" si="30"/>
         <v>5873.2383312876955</v>
       </c>
       <c r="S39" s="11">
-        <f>S24+S26-S30</f>
+        <f t="shared" si="30"/>
         <v>8924.3390825549795</v>
       </c>
       <c r="T39" s="11">
-        <f>T24+T26-T30</f>
+        <f t="shared" si="30"/>
         <v>11099.457576799137</v>
       </c>
     </row>
     <row r="40" spans="2:21" x14ac:dyDescent="0.3">
       <c r="B40" s="14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C40" s="14"/>
       <c r="D40" s="14"/>
-      <c r="E40" s="31">
-        <f>E39/E13</f>
+      <c r="E40" s="30">
+        <f t="shared" ref="E40:T40" si="31">E39/E13</f>
         <v>-3.1378496798112568E-2</v>
       </c>
-      <c r="F40" s="31">
-        <f>F39/F13</f>
+      <c r="F40" s="30">
+        <f t="shared" si="31"/>
         <v>9.6192640095130906E-3</v>
       </c>
-      <c r="G40" s="31">
-        <f>G39/G13</f>
+      <c r="G40" s="30">
+        <f t="shared" si="31"/>
         <v>0</v>
       </c>
-      <c r="H40" s="31">
-        <f>H39/H13</f>
+      <c r="H40" s="30">
+        <f t="shared" si="31"/>
         <v>0</v>
       </c>
-      <c r="I40" s="31">
-        <f>I39/I13</f>
+      <c r="I40" s="30">
+        <f t="shared" si="31"/>
         <v>-9.4893617021276597</v>
       </c>
-      <c r="J40" s="31">
-        <f>J39/J13</f>
+      <c r="J40" s="30">
+        <f t="shared" si="31"/>
         <v>-8.3389911328266386</v>
       </c>
-      <c r="K40" s="31">
-        <f>K39/K13</f>
+      <c r="K40" s="30">
+        <f t="shared" si="31"/>
         <v>-2.9072281595941649</v>
       </c>
-      <c r="L40" s="31">
-        <f>L39/L13</f>
-        <v>-1.0688991783395099</v>
-      </c>
-      <c r="M40" s="31">
-        <f>M39/M13</f>
-        <v>-0.64992367843206844</v>
-      </c>
-      <c r="N40" s="31">
-        <f>N39/N13</f>
-        <v>-0.27988850603391846</v>
-      </c>
-      <c r="O40" s="31">
-        <f>O39/O13</f>
-        <v>-0.13962873587485408</v>
-      </c>
-      <c r="P40" s="31">
-        <f>P39/P13</f>
-        <v>-5.4985862287368723E-2</v>
-      </c>
-      <c r="Q40" s="31">
-        <f>Q39/Q13</f>
-        <v>4.2140530313575959E-2</v>
-      </c>
-      <c r="R40" s="31">
-        <f>R39/R13</f>
+      <c r="L40" s="30">
+        <f t="shared" si="31"/>
+        <v>-1.0945197907412891</v>
+      </c>
+      <c r="M40" s="30">
+        <f t="shared" si="31"/>
+        <v>-0.6352372416296016</v>
+      </c>
+      <c r="N40" s="30">
+        <f t="shared" si="31"/>
+        <v>-0.31508850603391847</v>
+      </c>
+      <c r="O40" s="30">
+        <f t="shared" si="31"/>
+        <v>-0.16542873587485404</v>
+      </c>
+      <c r="P40" s="30">
+        <f t="shared" si="31"/>
+        <v>-7.1985862287368696E-2</v>
+      </c>
+      <c r="Q40" s="30">
+        <f t="shared" si="31"/>
+        <v>3.3640530313575959E-2</v>
+      </c>
+      <c r="R40" s="30">
+        <f t="shared" si="31"/>
         <v>0.10763333993030223</v>
       </c>
-      <c r="S40" s="31">
-        <f>S39/S13</f>
+      <c r="S40" s="30">
+        <f t="shared" si="31"/>
         <v>0.14868000611718929</v>
       </c>
-      <c r="T40" s="31">
-        <f>T39/T13</f>
+      <c r="T40" s="30">
+        <f t="shared" si="31"/>
         <v>0.17282019274722729</v>
       </c>
     </row>
     <row r="42" spans="2:21" x14ac:dyDescent="0.3">
-      <c r="B42" s="49" t="s">
-        <v>59</v>
-      </c>
-      <c r="C42" s="49"/>
-      <c r="D42" s="49"/>
-      <c r="E42" s="49"/>
-      <c r="F42" s="49" t="s">
-        <v>78</v>
-      </c>
-      <c r="G42" s="49"/>
-      <c r="H42" s="49"/>
-      <c r="I42" s="49"/>
-      <c r="J42" s="34"/>
-      <c r="K42" s="49" t="s">
-        <v>100</v>
-      </c>
-      <c r="L42" s="49"/>
-      <c r="M42" s="49"/>
-      <c r="N42" s="49"/>
-      <c r="O42" s="49" t="s">
-        <v>78</v>
-      </c>
-      <c r="P42" s="49"/>
-      <c r="Q42" s="49"/>
-      <c r="R42" s="49"/>
-      <c r="S42" s="49"/>
-      <c r="T42" s="49"/>
+      <c r="B42" s="45" t="s">
+        <v>58</v>
+      </c>
+      <c r="C42" s="45"/>
+      <c r="D42" s="45"/>
+      <c r="E42" s="45"/>
+      <c r="F42" s="45" t="s">
+        <v>77</v>
+      </c>
+      <c r="G42" s="45"/>
+      <c r="H42" s="45"/>
+      <c r="I42" s="45"/>
+      <c r="J42" s="33"/>
+      <c r="K42" s="45" t="s">
+        <v>98</v>
+      </c>
+      <c r="L42" s="45"/>
+      <c r="M42" s="45"/>
+      <c r="N42" s="45"/>
+      <c r="O42" s="45" t="s">
+        <v>77</v>
+      </c>
+      <c r="P42" s="45"/>
+      <c r="Q42" s="45"/>
+      <c r="R42" s="45"/>
+      <c r="S42" s="45"/>
+      <c r="T42" s="45"/>
     </row>
     <row r="43" spans="2:21" x14ac:dyDescent="0.3">
       <c r="B43" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E43" s="1">
         <v>22</v>
       </c>
       <c r="G43" s="14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I43" s="13"/>
       <c r="J43" s="13"/>
       <c r="K43" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="N43" s="37">
-        <v>0.03</v>
+        <v>82</v>
+      </c>
+      <c r="N43" s="36">
+        <v>2.5000000000000001E-2</v>
       </c>
     </row>
     <row r="44" spans="2:21" x14ac:dyDescent="0.3">
       <c r="B44" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E44" s="10">
         <v>1</v>
       </c>
       <c r="K44" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="N44" s="35">
+        <v>81</v>
+      </c>
+      <c r="N44" s="34">
         <f>(T39*(1+N43)/(E53-N43)) / (1 + E53)^10</f>
-        <v>46142.512891448423</v>
-      </c>
-      <c r="T44" s="44"/>
+        <v>43341.723246761925</v>
+      </c>
+      <c r="T44" s="43"/>
     </row>
     <row r="45" spans="2:21" x14ac:dyDescent="0.3">
       <c r="B45" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E45" s="10">
         <v>4.1300000000000003E-2</v>
       </c>
       <c r="G45" s="14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="46" spans="2:21" x14ac:dyDescent="0.3">
       <c r="B46" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E46" s="1">
         <v>1.1200000000000001</v>
       </c>
       <c r="K46" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="N46" s="35">
+        <v>83</v>
+      </c>
+      <c r="N46" s="34">
         <f>NPV(E53,K39:T39)</f>
-        <v>-22216.978306508954</v>
+        <v>-23882.569310254821</v>
       </c>
       <c r="P46" s="14" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="47" spans="2:21" x14ac:dyDescent="0.3">
       <c r="B47" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E47" s="10">
         <v>6.5000000000000002E-2</v>
@@ -2830,167 +2811,167 @@
     </row>
     <row r="48" spans="2:21" x14ac:dyDescent="0.3">
       <c r="B48" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E48" s="1">
         <v>4.0910000000000002</v>
       </c>
       <c r="G48" s="14" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="K48" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="N48" s="35">
+        <v>84</v>
+      </c>
+      <c r="N48" s="34">
         <f>N44+N46</f>
-        <v>23925.534584939469</v>
+        <v>19459.153936507104</v>
       </c>
     </row>
     <row r="49" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B49" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E49" s="10">
         <v>0</v>
       </c>
       <c r="K49" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="N49" s="35">
+        <v>90</v>
+      </c>
+      <c r="N49" s="34">
         <f>4000*0.75</f>
         <v>3000</v>
       </c>
       <c r="P49" s="14" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="50" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B50" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E50" s="10">
         <f>E45+E46*E47</f>
         <v>0.11410000000000001</v>
       </c>
       <c r="K50" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="N50" s="35">
+        <v>85</v>
+      </c>
+      <c r="N50" s="34">
         <f>1000*0.6</f>
         <v>600</v>
       </c>
       <c r="P50" s="14" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="51" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B51" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E51" s="10">
         <v>0.08</v>
       </c>
       <c r="K51" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="N51" s="35">
+        <v>86</v>
+      </c>
+      <c r="N51" s="34">
         <f>200*0.8</f>
         <v>160</v>
       </c>
       <c r="P51" s="14" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="52" spans="2:20" x14ac:dyDescent="0.3">
-      <c r="B52" s="36" t="s">
-        <v>52</v>
-      </c>
-      <c r="C52" s="36"/>
-      <c r="D52" s="36"/>
-      <c r="E52" s="39">
+      <c r="B52" s="35" t="s">
+        <v>51</v>
+      </c>
+      <c r="C52" s="35"/>
+      <c r="D52" s="35"/>
+      <c r="E52" s="38">
         <v>0.27</v>
       </c>
       <c r="K52" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="N52" s="35">
+        <v>87</v>
+      </c>
+      <c r="N52" s="34">
         <f>15000*0.28</f>
         <v>4200</v>
       </c>
       <c r="P52" s="14" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="53" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B53" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E53" s="10">
         <f>E44*E50+E49*E51*(1-E52)</f>
         <v>0.11410000000000001</v>
       </c>
-      <c r="K53" s="42" t="s">
-        <v>103</v>
-      </c>
-      <c r="L53" s="36"/>
-      <c r="M53" s="36"/>
-      <c r="N53" s="38">
+      <c r="K53" s="41" t="s">
+        <v>101</v>
+      </c>
+      <c r="L53" s="35"/>
+      <c r="M53" s="35"/>
+      <c r="N53" s="37">
         <f>N52+N51+N50+N49*0.7</f>
         <v>7060</v>
       </c>
       <c r="P53" s="14" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="54" spans="2:20" x14ac:dyDescent="0.3">
-      <c r="K54" s="41" t="s">
-        <v>105</v>
-      </c>
-      <c r="N54" s="35">
+      <c r="K54" s="40" t="s">
+        <v>103</v>
+      </c>
+      <c r="N54" s="34">
         <f>N53+N48</f>
-        <v>30985.534584939469</v>
+        <v>26519.153936507104</v>
       </c>
     </row>
     <row r="61" spans="2:20" x14ac:dyDescent="0.3">
       <c r="L61" s="1" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="63" spans="2:20" x14ac:dyDescent="0.3">
       <c r="J63" s="11">
-        <f t="shared" ref="J63:S63" si="23">K63-1</f>
+        <f t="shared" ref="J63:R63" si="32">K63-1</f>
         <v>0</v>
       </c>
       <c r="K63" s="11">
-        <f t="shared" si="23"/>
+        <f t="shared" si="32"/>
         <v>1</v>
       </c>
       <c r="L63" s="11">
-        <f t="shared" si="23"/>
+        <f t="shared" si="32"/>
         <v>2</v>
       </c>
       <c r="M63" s="11">
-        <f t="shared" si="23"/>
+        <f t="shared" si="32"/>
         <v>3</v>
       </c>
       <c r="N63" s="11">
-        <f t="shared" si="23"/>
+        <f t="shared" si="32"/>
         <v>4</v>
       </c>
       <c r="O63" s="11">
-        <f t="shared" si="23"/>
+        <f t="shared" si="32"/>
         <v>5</v>
       </c>
       <c r="P63" s="11">
-        <f t="shared" si="23"/>
+        <f t="shared" si="32"/>
         <v>6</v>
       </c>
       <c r="Q63" s="11">
-        <f t="shared" si="23"/>
+        <f t="shared" si="32"/>
         <v>7</v>
       </c>
       <c r="R63" s="11">
-        <f t="shared" si="23"/>
+        <f t="shared" si="32"/>
         <v>8</v>
       </c>
       <c r="S63" s="11">
@@ -3003,6 +2984,23 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="B2:C4"/>
+    <mergeCell ref="D2:F4"/>
+    <mergeCell ref="H6:M6"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="O6:Q6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B42:E42"/>
+    <mergeCell ref="F42:I42"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="H11:I11"/>
     <mergeCell ref="K42:N42"/>
     <mergeCell ref="D10:F10"/>
     <mergeCell ref="D11:F11"/>
@@ -3016,23 +3014,6 @@
     <mergeCell ref="D9:F9"/>
     <mergeCell ref="O42:T42"/>
     <mergeCell ref="J11:M11"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B42:E42"/>
-    <mergeCell ref="F42:I42"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="B2:C4"/>
-    <mergeCell ref="D2:F4"/>
-    <mergeCell ref="H6:M6"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="O6:Q6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -3071,7 +3052,7 @@
     <row r="2" spans="1:20" s="58" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="58" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:20" s="58" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -3093,46 +3074,46 @@
     </row>
     <row r="5" spans="1:20" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G5" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="H5" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="I5" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="J5" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="J5" s="3" t="s">
+      <c r="K5" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="K5" s="3" t="s">
+      <c r="L5" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="L5" s="3" t="s">
+      <c r="M5" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="M5" s="3" t="s">
+      <c r="N5" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="N5" s="3" t="s">
+      <c r="O5" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="O5" s="3" t="s">
-        <v>39</v>
-      </c>
       <c r="P5" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q5" s="3" t="s">
         <v>45</v>
-      </c>
-      <c r="Q5" s="3" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:20" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -3151,7 +3132,7 @@
     </row>
     <row r="7" spans="1:20" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="13" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E7" s="11"/>
       <c r="F7" s="11">
@@ -3204,7 +3185,7 @@
     </row>
     <row r="8" spans="1:20" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E8" s="11"/>
       <c r="F8" s="11">
@@ -3256,7 +3237,7 @@
     </row>
     <row r="9" spans="1:20" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E9" s="11"/>
       <c r="F9" s="11">
@@ -3310,7 +3291,7 @@
     </row>
     <row r="10" spans="1:20" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C10" s="6"/>
       <c r="D10" s="6"/>
@@ -3393,7 +3374,7 @@
     </row>
     <row r="13" spans="1:20" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E13" s="11"/>
       <c r="F13" s="11">
@@ -3435,7 +3416,7 @@
     </row>
     <row r="14" spans="1:20" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E14" s="11"/>
       <c r="F14" s="11">
@@ -3477,7 +3458,7 @@
     </row>
     <row r="15" spans="1:20" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E15" s="11"/>
       <c r="F15" s="11">
@@ -3531,7 +3512,7 @@
     </row>
     <row r="16" spans="1:20" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="14" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C16" s="14"/>
       <c r="D16" s="14"/>
@@ -3587,7 +3568,7 @@
     </row>
     <row r="17" spans="2:19" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E17" s="11"/>
       <c r="F17" s="7"/>
@@ -3641,7 +3622,7 @@
     </row>
     <row r="19" spans="2:19" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E19" s="11"/>
       <c r="F19" s="11">
@@ -3683,7 +3664,7 @@
     </row>
     <row r="20" spans="2:19" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E20" s="11"/>
       <c r="F20" s="11">
@@ -3752,7 +3733,7 @@
     </row>
     <row r="22" spans="2:19" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E22" s="11"/>
       <c r="F22" s="11">
@@ -3794,7 +3775,7 @@
     </row>
     <row r="23" spans="2:19" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F23" s="11">
         <v>0</v>
@@ -3835,7 +3816,7 @@
     </row>
     <row r="24" spans="2:19" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E24" s="11"/>
       <c r="F24" s="11">
@@ -3904,7 +3885,7 @@
     </row>
     <row r="26" spans="2:19" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F26" s="11">
         <v>9</v>
@@ -3945,7 +3926,7 @@
     </row>
     <row r="27" spans="2:19" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F27" s="7">
         <v>0</v>
@@ -4013,7 +3994,7 @@
     </row>
     <row r="29" spans="2:19" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B29" s="13" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F29" s="11">
         <f t="shared" ref="F29:N29" si="9">F24-F26</f>
@@ -4066,7 +4047,7 @@
     </row>
     <row r="30" spans="2:19" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C30" s="6"/>
       <c r="D30" s="6"/>
@@ -4123,7 +4104,7 @@
     </row>
     <row r="32" spans="2:19" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F32" s="11">
         <v>-13730</v>
@@ -4164,7 +4145,7 @@
     </row>
     <row r="33" spans="2:17" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B33" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F33" s="11"/>
       <c r="G33" s="11"/>

</xml_diff>